<commit_message>
Update ils-postplanner-2026-06-02.xlsx (regenerated during June 3 pipeline run)
</commit_message>
<xml_diff>
--- a/Softball/postplanner-imports/ils-postplanner-2026-06-02.xlsx
+++ b/Softball/postplanner-imports/ils-postplanner-2026-06-02.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/02/2026  10:50</t>
+          <t>06/02/2026  09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06/02/2026  12:20</t>
+          <t>06/02/2026  09:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,7 +508,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06/02/2026  13:50</t>
+          <t>06/02/2026  11:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -524,7 +524,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06/02/2026  15:20</t>
+          <t>06/02/2026  11:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -540,7 +540,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/02/2026  16:50</t>
+          <t>06/02/2026  13:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -556,7 +556,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/02/2026  18:20</t>
+          <t>06/02/2026  15:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06/02/2026  19:50</t>
+          <t>06/02/2026  17:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">

</xml_diff>